<commit_message>
HDPI-7052: add header rows to GroupAccess tabs
</commit_message>
<xml_diff>
--- a/data/ccd-template.xlsx
+++ b/data/ccd-template.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/taleb/projects/reform/repos/ccd-definition-processor/data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/taleb/projects/reform/repos/coe/ccd-definition-processor/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D318551A-C44E-7442-A777-B9AA1C62E173}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4384F709-2700-3A4F-9559-62008591CCAE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="780" windowWidth="36000" windowHeight="22600" tabRatio="500" firstSheet="20" activeTab="30" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="780" windowWidth="36000" windowHeight="21040" tabRatio="500" firstSheet="20" activeTab="30" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Jurisdiction" sheetId="1" r:id="rId1"/>
@@ -55,7 +55,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="611" uniqueCount="265">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="661" uniqueCount="291">
   <si>
     <t>Jurisdiction</t>
   </si>
@@ -942,6 +942,96 @@
   </si>
   <si>
     <t>ParentCategoryID</t>
+  </si>
+  <si>
+    <t>AccessType</t>
+  </si>
+  <si>
+    <t>PrimaryKeyIn Red</t>
+  </si>
+  <si>
+    <t>The identifier which defines the accesstype code
+MaxLength: 200</t>
+  </si>
+  <si>
+    <t>This can be a CCD base type (see confluence) or a OrganisationProfile ID).  
+MaxLength: 200</t>
+  </si>
+  <si>
+    <t>Access type is mandatory for the given organisation type. (YesOrNo field Optional)</t>
+  </si>
+  <si>
+    <t>Field that indicates whether this access is applied by default for the given organisation type.
+If no specific configuration has been provided for a user (either to explicitly enable or disable the accesstype), this determines whether the user receives the access type by default.
+(YesOrNo field Optional)</t>
+  </si>
+  <si>
+    <t>Field that Indicates whether this access type is displayed to the user in the Invite User / Edit User UI.
+(YesOrNo field Optional)</t>
+  </si>
+  <si>
+    <t>The long description to decribe the access type.
+MaxLength: 200</t>
+  </si>
+  <si>
+    <t>The hint text that is present for this access type
+MaxLength: 300</t>
+  </si>
+  <si>
+    <t>The Order access types are displayed in UI</t>
+  </si>
+  <si>
+    <t>AccessTypeID</t>
+  </si>
+  <si>
+    <t>OrganisationProfileID</t>
+  </si>
+  <si>
+    <t>AccessMandatory</t>
+  </si>
+  <si>
+    <t>AccessDefault</t>
+  </si>
+  <si>
+    <t>Display</t>
+  </si>
+  <si>
+    <t>AccessTypeRole</t>
+  </si>
+  <si>
+    <t>The role name that is used to create organisation role assignments for this record.
+MaxLength: 70</t>
+  </si>
+  <si>
+    <t>The role name that is used to create access role assignments for this record.
+MaxLength: 70</t>
+  </si>
+  <si>
+    <t>This field uniquely identifies the OrganisationPolicy.
+MaxLength: 70</t>
+  </si>
+  <si>
+    <t>Indicates whether this record is active for group access.
+(YesOrNo field Optional)</t>
+  </si>
+  <si>
+    <t>A text template used to generate the case access group identifier for role assignments and case data.
+MaxLength: 200</t>
+  </si>
+  <si>
+    <t>OrganisationalRoleName</t>
+  </si>
+  <si>
+    <t>GroupRoleName</t>
+  </si>
+  <si>
+    <t>CaseAssignedRoleField</t>
+  </si>
+  <si>
+    <t>GroupAccessEnabled</t>
+  </si>
+  <si>
+    <t>CaseAccessGroupIDTemplate</t>
   </si>
 </sst>
 </file>
@@ -953,7 +1043,7 @@
     <numFmt numFmtId="165" formatCode="m/d/yyyy"/>
     <numFmt numFmtId="166" formatCode="dd/mm/yy"/>
   </numFmts>
-  <fonts count="36" x14ac:knownFonts="1">
+  <fonts count="44" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color rgb="FF000000"/>
@@ -1217,8 +1307,57 @@
       <family val="2"/>
       <charset val="1"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF984807"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color theme="0"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="14"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FFFF0000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FFFFC000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1231,8 +1370,20 @@
         <bgColor rgb="FF0000FF"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF0432FF"/>
+        <bgColor rgb="FF0432FF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+        <bgColor auto="1"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="7">
+  <borders count="11">
     <border>
       <left/>
       <right/>
@@ -1322,12 +1473,72 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color theme="1"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color theme="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="1"/>
+      </left>
+      <right style="thin">
+        <color theme="1"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color theme="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="1"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color theme="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="89">
+  <cellXfs count="102">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
@@ -1462,6 +1673,35 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="165" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="37" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="39" fillId="3" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="39" fillId="3" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="40" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="49" fontId="41" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="49" fontId="42" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="49" fontId="36" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="38" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="49" fontId="43" fillId="3" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="43" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -3478,8 +3718,11 @@
   <dimension ref="A1:F3"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="2" width="10.6640625" style="1" customWidth="1"/>
-    <col min="3" max="1025" width="10.5" customWidth="1"/>
+    <col min="1" max="1" width="28.83203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.5" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="25.5" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.33203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="1025" width="10.5" customWidth="1"/>
     <col min="16384" max="16384" width="9.33203125" customWidth="1"/>
   </cols>
   <sheetData>
@@ -3553,7 +3796,11 @@
   <dimension ref="A1:G3"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1025" width="10.5" customWidth="1"/>
+    <col min="1" max="1" width="33.1640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="25.5" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.33203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="1025" width="10.5" customWidth="1"/>
     <col min="16384" max="16384" width="9.33203125" customWidth="1"/>
   </cols>
   <sheetData>
@@ -6815,18 +7062,214 @@
 
 <file path=xl/worksheets/sheet30.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F4D20F22-26A3-ED45-BE50-60F3BDD1D8FC}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:K3"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="14" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="25.5" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.33203125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="12" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:11" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="95" t="s">
+        <v>265</v>
+      </c>
+      <c r="B1" s="96" t="s">
+        <v>266</v>
+      </c>
+      <c r="C1" s="97" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="98" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="99"/>
+      <c r="F1" s="99"/>
+      <c r="G1" s="99"/>
+      <c r="H1" s="99"/>
+      <c r="I1" s="99"/>
+      <c r="J1" s="99"/>
+      <c r="K1" s="99"/>
+    </row>
+    <row r="2" spans="1:11" ht="168" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="89" t="s">
+        <v>4</v>
+      </c>
+      <c r="B2" s="89" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2" s="89" t="s">
+        <v>6</v>
+      </c>
+      <c r="D2" s="89" t="s">
+        <v>267</v>
+      </c>
+      <c r="E2" s="89" t="s">
+        <v>268</v>
+      </c>
+      <c r="F2" s="89" t="s">
+        <v>269</v>
+      </c>
+      <c r="G2" s="89" t="s">
+        <v>270</v>
+      </c>
+      <c r="H2" s="90" t="s">
+        <v>271</v>
+      </c>
+      <c r="I2" s="89" t="s">
+        <v>272</v>
+      </c>
+      <c r="J2" s="89" t="s">
+        <v>273</v>
+      </c>
+      <c r="K2" s="91" t="s">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A3" s="92" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3" s="93" t="s">
+        <v>11</v>
+      </c>
+      <c r="C3" s="93" t="s">
+        <v>19</v>
+      </c>
+      <c r="D3" s="93" t="s">
+        <v>275</v>
+      </c>
+      <c r="E3" s="93" t="s">
+        <v>276</v>
+      </c>
+      <c r="F3" s="93" t="s">
+        <v>277</v>
+      </c>
+      <c r="G3" s="93" t="s">
+        <v>278</v>
+      </c>
+      <c r="H3" s="93" t="s">
+        <v>279</v>
+      </c>
+      <c r="I3" s="93" t="s">
+        <v>14</v>
+      </c>
+      <c r="J3" s="93" t="s">
+        <v>75</v>
+      </c>
+      <c r="K3" s="94" t="s">
+        <v>153</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet31.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9869F684-9B4A-FD42-95B4-C508556C4002}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:J3"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="19" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="25.5" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.33203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="18.83203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="21.83203125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.5" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="20.83203125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="19.1640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="26" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:10" ht="18" x14ac:dyDescent="0.2">
+      <c r="A1" s="95" t="s">
+        <v>280</v>
+      </c>
+      <c r="B1" s="96" t="s">
+        <v>266</v>
+      </c>
+      <c r="C1" s="97" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="98" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="99"/>
+      <c r="F1" s="99"/>
+      <c r="G1" s="99"/>
+      <c r="H1" s="99"/>
+      <c r="I1" s="99"/>
+      <c r="J1" s="99"/>
+    </row>
+    <row r="2" spans="1:10" ht="197" x14ac:dyDescent="0.2">
+      <c r="A2" s="89" t="s">
+        <v>4</v>
+      </c>
+      <c r="B2" s="89" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2" s="89" t="s">
+        <v>6</v>
+      </c>
+      <c r="D2" s="89" t="s">
+        <v>267</v>
+      </c>
+      <c r="E2" s="89" t="s">
+        <v>268</v>
+      </c>
+      <c r="F2" s="91" t="s">
+        <v>281</v>
+      </c>
+      <c r="G2" s="91" t="s">
+        <v>282</v>
+      </c>
+      <c r="H2" s="89" t="s">
+        <v>283</v>
+      </c>
+      <c r="I2" s="90" t="s">
+        <v>284</v>
+      </c>
+      <c r="J2" s="90" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A3" s="100" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3" s="100" t="s">
+        <v>11</v>
+      </c>
+      <c r="C3" s="100" t="s">
+        <v>19</v>
+      </c>
+      <c r="D3" s="100" t="s">
+        <v>275</v>
+      </c>
+      <c r="E3" s="100" t="s">
+        <v>276</v>
+      </c>
+      <c r="F3" s="101" t="s">
+        <v>286</v>
+      </c>
+      <c r="G3" s="100" t="s">
+        <v>287</v>
+      </c>
+      <c r="H3" s="100" t="s">
+        <v>288</v>
+      </c>
+      <c r="I3" s="100" t="s">
+        <v>289</v>
+      </c>
+      <c r="J3" s="100" t="s">
+        <v>290</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
HDPI-7052: adjust liveFrom/liveTo column types for GroupAccess tabs
</commit_message>
<xml_diff>
--- a/data/ccd-template.xlsx
+++ b/data/ccd-template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/taleb/projects/reform/repos/coe/ccd-definition-processor/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4384F709-2700-3A4F-9559-62008591CCAE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F6FA0DD-A774-E84A-8C01-82F4E47EFB39}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="780" windowWidth="36000" windowHeight="21040" tabRatio="500" firstSheet="20" activeTab="30" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="780" windowWidth="36000" windowHeight="21040" tabRatio="500" firstSheet="20" activeTab="29" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Jurisdiction" sheetId="1" r:id="rId1"/>
@@ -1538,7 +1538,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="102">
+  <cellXfs count="104">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
@@ -1683,9 +1683,6 @@
     <xf numFmtId="0" fontId="37" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="39" fillId="3" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="49" fontId="39" fillId="3" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -1701,6 +1698,15 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="43" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="43" fillId="3" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="3" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="3" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -7073,25 +7079,25 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="95" t="s">
+      <c r="A1" s="94" t="s">
         <v>265</v>
       </c>
-      <c r="B1" s="96" t="s">
+      <c r="B1" s="95" t="s">
         <v>266</v>
       </c>
-      <c r="C1" s="97" t="s">
+      <c r="C1" s="96" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="98" t="s">
+      <c r="D1" s="97" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="99"/>
-      <c r="F1" s="99"/>
-      <c r="G1" s="99"/>
-      <c r="H1" s="99"/>
-      <c r="I1" s="99"/>
-      <c r="J1" s="99"/>
-      <c r="K1" s="99"/>
+      <c r="E1" s="98"/>
+      <c r="F1" s="98"/>
+      <c r="G1" s="98"/>
+      <c r="H1" s="98"/>
+      <c r="I1" s="98"/>
+      <c r="J1" s="98"/>
+      <c r="K1" s="98"/>
     </row>
     <row r="2" spans="1:11" ht="168" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="89" t="s">
@@ -7129,37 +7135,37 @@
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A3" s="92" t="s">
+      <c r="A3" s="102" t="s">
         <v>10</v>
       </c>
-      <c r="B3" s="93" t="s">
+      <c r="B3" s="103" t="s">
         <v>11</v>
       </c>
-      <c r="C3" s="93" t="s">
+      <c r="C3" s="92" t="s">
         <v>19</v>
       </c>
-      <c r="D3" s="93" t="s">
+      <c r="D3" s="92" t="s">
         <v>275</v>
       </c>
-      <c r="E3" s="93" t="s">
+      <c r="E3" s="92" t="s">
         <v>276</v>
       </c>
-      <c r="F3" s="93" t="s">
+      <c r="F3" s="92" t="s">
         <v>277</v>
       </c>
-      <c r="G3" s="93" t="s">
+      <c r="G3" s="92" t="s">
         <v>278</v>
       </c>
-      <c r="H3" s="93" t="s">
+      <c r="H3" s="92" t="s">
         <v>279</v>
       </c>
-      <c r="I3" s="93" t="s">
+      <c r="I3" s="92" t="s">
         <v>14</v>
       </c>
-      <c r="J3" s="93" t="s">
+      <c r="J3" s="92" t="s">
         <v>75</v>
       </c>
-      <c r="K3" s="94" t="s">
+      <c r="K3" s="93" t="s">
         <v>153</v>
       </c>
     </row>
@@ -7186,26 +7192,26 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="18" x14ac:dyDescent="0.2">
-      <c r="A1" s="95" t="s">
+      <c r="A1" s="94" t="s">
         <v>280</v>
       </c>
-      <c r="B1" s="96" t="s">
+      <c r="B1" s="95" t="s">
         <v>266</v>
       </c>
-      <c r="C1" s="97" t="s">
+      <c r="C1" s="96" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="98" t="s">
+      <c r="D1" s="97" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="99"/>
-      <c r="F1" s="99"/>
-      <c r="G1" s="99"/>
-      <c r="H1" s="99"/>
-      <c r="I1" s="99"/>
-      <c r="J1" s="99"/>
-    </row>
-    <row r="2" spans="1:10" ht="197" x14ac:dyDescent="0.2">
+      <c r="E1" s="98"/>
+      <c r="F1" s="98"/>
+      <c r="G1" s="98"/>
+      <c r="H1" s="98"/>
+      <c r="I1" s="98"/>
+      <c r="J1" s="98"/>
+    </row>
+    <row r="2" spans="1:10" ht="85" x14ac:dyDescent="0.2">
       <c r="A2" s="89" t="s">
         <v>4</v>
       </c>
@@ -7238,34 +7244,34 @@
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A3" s="100" t="s">
+      <c r="A3" s="101" t="s">
         <v>10</v>
       </c>
-      <c r="B3" s="100" t="s">
+      <c r="B3" s="101" t="s">
         <v>11</v>
       </c>
-      <c r="C3" s="100" t="s">
+      <c r="C3" s="99" t="s">
         <v>19</v>
       </c>
-      <c r="D3" s="100" t="s">
+      <c r="D3" s="99" t="s">
         <v>275</v>
       </c>
-      <c r="E3" s="100" t="s">
+      <c r="E3" s="99" t="s">
         <v>276</v>
       </c>
-      <c r="F3" s="101" t="s">
+      <c r="F3" s="100" t="s">
         <v>286</v>
       </c>
-      <c r="G3" s="100" t="s">
+      <c r="G3" s="99" t="s">
         <v>287</v>
       </c>
-      <c r="H3" s="100" t="s">
+      <c r="H3" s="99" t="s">
         <v>288</v>
       </c>
-      <c r="I3" s="100" t="s">
+      <c r="I3" s="99" t="s">
         <v>289</v>
       </c>
-      <c r="J3" s="100" t="s">
+      <c r="J3" s="99" t="s">
         <v>290</v>
       </c>
     </row>

</xml_diff>